<commit_message>
Model VM sizing from TTS throughput and default PG reserved pricing
</commit_message>
<xml_diff>
--- a/exports/costs/azure-cost-model.xlsx
+++ b/exports/costs/azure-cost-model.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="230">
   <si>
     <t>Workbook</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-02-10T02:32:00.057Z</t>
+    <t>2026-02-10T02:48:19.738Z</t>
   </si>
   <si>
     <t>Region</t>
@@ -329,6 +329,27 @@
     <t>USD/month</t>
   </si>
   <si>
+    <t>Capacity knobs</t>
+  </si>
+  <si>
+    <t>Kokoro real-time factor per VM</t>
+  </si>
+  <si>
+    <t>x realtime</t>
+  </si>
+  <si>
+    <t>Target VM utilization</t>
+  </si>
+  <si>
+    <t>Web/API overhead fraction</t>
+  </si>
+  <si>
+    <t>API submissions capacity per VM hour</t>
+  </si>
+  <si>
+    <t>submissions/hour</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -392,6 +413,39 @@
     <t>effective jobs * ops/article</t>
   </si>
   <si>
+    <t>Peak submissions / hour</t>
+  </si>
+  <si>
+    <t>(users/1000) * peak_submissions_per_1000 * scenario usage multiplier</t>
+  </si>
+  <si>
+    <t>TTS capacity minutes / VM / month</t>
+  </si>
+  <si>
+    <t>hours * 60 * realtime_factor * utilization * (1-overhead)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Required VMs (TTS)</t>
+  </si>
+  <si>
+    <t>ceil(audio_minutes / tts_capacity_per_vm)</t>
+  </si>
+  <si>
+    <t>Required VMs (API peak)</t>
+  </si>
+  <si>
+    <t>ceil((peak_submissions_hour * headroom)/api_capacity_per_vm_hour)</t>
+  </si>
+  <si>
+    <t>Required VMs (total)</t>
+  </si>
+  <si>
+    <t>max(base_vm_count, vm_tts, vm_api)</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
@@ -473,7 +527,7 @@
     <t>VM compute</t>
   </si>
   <si>
-    <t>vm_hourly * hours * vm_count</t>
+    <t>vm_hourly * hours * required_vm_count</t>
   </si>
   <si>
     <t>VM public IP</t>
@@ -491,7 +545,7 @@
     <t>Postgres compute</t>
   </si>
   <si>
-    <t>pg_vcore_hourly * vcores * hours</t>
+    <t>pg_vcore_3yr_reserved * vcores / 36</t>
   </si>
   <si>
     <t>pg_storage_rate * 128GB</t>
@@ -600,6 +654,24 @@
   </si>
   <si>
     <t>USD/year</t>
+  </si>
+  <si>
+    <t>Estimated required VM count</t>
+  </si>
+  <si>
+    <t>Computed from TTS + API peak</t>
+  </si>
+  <si>
+    <t>Required VMs for TTS only</t>
+  </si>
+  <si>
+    <t>Capacity from Kokoro realtime factor</t>
+  </si>
+  <si>
+    <t>Required VMs for API peak only</t>
+  </si>
+  <si>
+    <t>Headroom-adjusted request peak</t>
   </si>
   <si>
     <t>Best commitment monthly</t>
@@ -1115,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1859,6 +1931,76 @@
       </c>
       <c r="D48" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>103</v>
+      </c>
+      <c r="B51" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="D51" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C52" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="D52" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>103</v>
+      </c>
+      <c r="B53" t="s">
+        <v>107</v>
+      </c>
+      <c r="C53" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D53" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>103</v>
+      </c>
+      <c r="B54" t="s">
+        <v>108</v>
+      </c>
+      <c r="C54" s="2">
+        <v>120</v>
+      </c>
+      <c r="D54" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +2016,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1885,10 +2027,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>41</v>
@@ -1900,15 +2042,15 @@
         <v>43</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C2" s="3">
         <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C13*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))*Inputs!C3</f>
@@ -1925,10 +2067,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C3" s="3">
         <f>C2*(1+Inputs!C8)</f>
@@ -1945,10 +2087,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C4" s="3">
         <f>C3*Inputs!C7</f>
@@ -1965,10 +2107,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="C5" s="3">
         <f>C4*Inputs!C15*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
@@ -1985,10 +2127,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C6" s="3">
         <f>(C5*Inputs!C20)/1024</f>
@@ -2005,10 +2147,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C7" s="3">
         <f>C4*Inputs!C21</f>
@@ -2025,10 +2167,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C8" s="3">
         <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C22*IF(Inputs!C2="Low",Inputs!E28,IF(Inputs!C2="High",Inputs!E30,Inputs!E29))</f>
@@ -2045,10 +2187,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C9" s="3">
         <f>(C3*Inputs!C24)/(1024*1024)</f>
@@ -2065,10 +2207,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="C10" s="3">
         <f>C3*Inputs!C25</f>
@@ -2081,6 +2223,106 @@
       </c>
       <c r="F10" s="3">
         <f>SUM(C10:E10)</f>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="3">
+        <f>(Inputs!C12/1000)*Inputs!C14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+      </c>
+      <c r="D11" s="3">
+        <f>(Inputs!D12/1000)*Inputs!D14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+      </c>
+      <c r="E11" s="3">
+        <f>(Inputs!E12/1000)*Inputs!E14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+      </c>
+      <c r="F11" s="3">
+        <f>SUM(C11:E11)</f>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" t="s">
+        <v>135</v>
+      </c>
+      <c r="F12" s="3">
+        <f>Inputs!C4*60*Inputs!C51*Inputs!C52*(1-Inputs!C53)</f>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" t="s">
+        <v>135</v>
+      </c>
+      <c r="D13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" t="s">
+        <v>135</v>
+      </c>
+      <c r="F13" s="3">
+        <f>MAX(1,ROUNDUP(F5/F12,0))</f>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" t="s">
+        <v>135</v>
+      </c>
+      <c r="F14" s="3">
+        <f>MAX(1,ROUNDUP((F11*Inputs!C5)/Inputs!C54,0))</f>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" t="s">
+        <v>135</v>
+      </c>
+      <c r="D15" t="s">
+        <v>135</v>
+      </c>
+      <c r="E15" t="s">
+        <v>135</v>
+      </c>
+      <c r="F15" s="3">
+        <f>MAX(Inputs!C6,F13,F14)</f>
       </c>
     </row>
   </sheetData>
@@ -2103,24 +2345,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B2" t="s">
         <v>81</v>
@@ -2137,10 +2379,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B3" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="C3">
         <v>889</v>
@@ -2154,10 +2396,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="C4">
         <v>1718</v>
@@ -2171,10 +2413,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B5" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C5">
         <v>0.089</v>
@@ -2188,10 +2430,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B6" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="C6">
         <v>468</v>
@@ -2205,10 +2447,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B7" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
       <c r="C7">
         <v>936</v>
@@ -2222,10 +2464,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="C8">
         <v>0.115</v>
@@ -2239,10 +2481,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="C9">
         <v>0.095</v>
@@ -2256,10 +2498,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="B10" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="C10">
         <v>0.0208</v>
@@ -2273,16 +2515,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="B11" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="C11">
         <v>0.05</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="E11" t="s">
         <v>3</v>
@@ -2290,16 +2532,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="C12">
         <v>0.004</v>
       </c>
       <c r="D12" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="E12" t="s">
         <v>3</v>
@@ -2310,7 +2552,7 @@
         <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="C13">
         <v>0.045</v>
@@ -2327,13 +2569,13 @@
         <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="C14">
         <v>0.00036</v>
       </c>
       <c r="D14" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="E14" t="s">
         <v>3</v>
@@ -2361,7 +2603,7 @@
         <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="C16">
         <v>0.005</v>
@@ -2375,10 +2617,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="B17" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="C17">
         <v>5.2795</v>
@@ -2409,33 +2651,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="C2" s="3">
-        <f>Inputs!C33*Inputs!C4*Inputs!C6</f>
+        <f>Inputs!C33*Inputs!C4*Formulas!F15</f>
       </c>
       <c r="D2" s="3">
-        <f>Inputs!C33*Inputs!C4*Inputs!C6*12</f>
+        <f>Inputs!C33*Inputs!C4*Formulas!F15*12</f>
       </c>
       <c r="E2" s="3">
         <f>C2/SUM(C2:C13)</f>
@@ -2443,10 +2685,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="C3" s="3">
         <f>Inputs!C47*Inputs!C4</f>
@@ -2460,10 +2702,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="B4" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="C4" s="3">
         <f>Inputs!C48</f>
@@ -2477,16 +2719,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="B5" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="C5" s="3">
-        <f>Inputs!C36*2*Inputs!C4</f>
+        <f>(Inputs!C38/36)*2</f>
       </c>
       <c r="D5" s="3">
-        <f>Inputs!C36*2*Inputs!C4*12</f>
+        <f>(Inputs!C38/36)*2*12</f>
       </c>
       <c r="E5" s="3">
         <f>C5/SUM(C2:C13)</f>
@@ -2497,7 +2739,7 @@
         <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="C6" s="3">
         <f>Inputs!C39*128</f>
@@ -2511,10 +2753,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="B7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="C7" s="3">
         <f>Inputs!C40*128*Inputs!C9</f>
@@ -2528,10 +2770,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="B8" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="C8" s="3">
         <f>Inputs!C41*MAX(128,Formulas!F6*3)</f>
@@ -2548,7 +2790,7 @@
         <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="C9" s="3">
         <f>Inputs!C42*(Formulas!F4/10000)</f>
@@ -2565,7 +2807,7 @@
         <v>95</v>
       </c>
       <c r="B10" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="C10" s="3">
         <f>Inputs!C43*(Formulas!F7/10000)</f>
@@ -2579,10 +2821,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="B11" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="C11" s="3">
         <f>Inputs!C44*MAX(5,Formulas!F9*2)</f>
@@ -2599,7 +2841,7 @@
         <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="C12" s="3">
         <f>Inputs!C45*(Formulas!F10/10000)</f>
@@ -2613,10 +2855,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="B13" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="C13" s="3">
         <f>Inputs!C46*Formulas!F8</f>
@@ -2630,10 +2872,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="C14" s="1">
         <f>SUM(C2:C13)</f>
@@ -2642,7 +2884,7 @@
         <f>SUM(D2:D13)</f>
       </c>
       <c r="E14" s="1" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2663,24 +2905,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="B2" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -2697,41 +2939,41 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="B3" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Inputs!C6</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15</f>
       </c>
       <c r="C3" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Inputs!C6*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15*12</f>
       </c>
       <c r="D3" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Inputs!C6)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15)</f>
       </c>
       <c r="E3" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Inputs!C6))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15))/B2)</f>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="B4" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Inputs!C6</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15</f>
       </c>
       <c r="C4" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Inputs!C6*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15*12</f>
       </c>
       <c r="D4" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Inputs!C6)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15)</f>
       </c>
       <c r="E4" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Inputs!C6))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15))/B2)</f>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="B5" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2</f>
@@ -2748,7 +2990,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="B6" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2</f>
@@ -2765,36 +3007,36 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="B7" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Inputs!C6 + (Inputs!C37/12)*2</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2</f>
       </c>
       <c r="C7" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Inputs!C6 + (Inputs!C37/12)*2*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2*12</f>
       </c>
       <c r="D7" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Inputs!C6 + (Inputs!C37/12)*2)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2)</f>
       </c>
       <c r="E7" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Inputs!C6 + (Inputs!C37/12)*2))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2))/B2)</f>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="B8" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Inputs!C6 + (Inputs!C38/36)*2</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2</f>
       </c>
       <c r="C8" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Inputs!C6 + (Inputs!C38/36)*2*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2*12</f>
       </c>
       <c r="D8" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Inputs!C6 + (Inputs!C38/36)*2)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2)</f>
       </c>
       <c r="E8" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Inputs!C6 + (Inputs!C38/36)*2))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2))/B2)</f>
       </c>
     </row>
   </sheetData>
@@ -2815,16 +3057,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2843,7 +3085,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
       <c r="B3">
         <v>0.75</v>
@@ -2857,7 +3099,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="B4">
         <v>1.25</v>
@@ -2871,7 +3113,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="B5">
         <v>1.5</v>
@@ -2891,7 +3133,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2900,29 +3142,29 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="B2" s="3">
         <f>Inputs!C2</f>
       </c>
       <c r="C2" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>191</v>
+        <v>209</v>
       </c>
       <c r="B3" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -2933,68 +3175,101 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="B4" s="3">
         <f>Cost_Breakdown!D14</f>
       </c>
       <c r="C4" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="B5" s="3">
-        <f>MIN(Commitment_Compare!B2:B8)</f>
+        <f>Formulas!F15</f>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>196</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>181</v>
+        <v>214</v>
+      </c>
+      <c r="B6" s="3">
+        <f>Formulas!F13</f>
       </c>
       <c r="C6" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>198</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>199</v>
+        <v>216</v>
+      </c>
+      <c r="B7" s="3">
+        <f>Formulas!F14</f>
       </c>
       <c r="C7" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>201</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>202</v>
+        <v>218</v>
+      </c>
+      <c r="B8" s="3">
+        <f>MIN(Commitment_Compare!B2:B8)</f>
       </c>
       <c r="C8" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>222</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C11" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>228</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C9" t="s">
-        <v>205</v>
+      <c r="C12" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 90/95 margin pricing calculator to Azure cost model
</commit_message>
<xml_diff>
--- a/exports/costs/azure-cost-model.xlsx
+++ b/exports/costs/azure-cost-model.xlsx
@@ -10,15 +10,16 @@
     <sheet sheetId="4" name="Prices" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Cost_Breakdown" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Commitment_Compare" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Sensitivity" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Finance_Summary" state="visible" r:id="rId11"/>
+    <sheet sheetId="7" name="Pricing_Strategy" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Sensitivity" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Finance_Summary" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="265">
   <si>
     <t>Workbook</t>
   </si>
@@ -29,7 +30,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-02-10T02:48:19.738Z</t>
+    <t>2026-02-10T02:52:00.477Z</t>
   </si>
   <si>
     <t>Region</t>
@@ -350,6 +351,18 @@
     <t>submissions/hour</t>
   </si>
   <si>
+    <t>Pricing knobs</t>
+  </si>
+  <si>
+    <t>Target gross margin (floor)</t>
+  </si>
+  <si>
+    <t>Target gross margin (comfort)</t>
+  </si>
+  <si>
+    <t>Team price multiplier vs Pro</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -620,6 +633,84 @@
     <t>VM + Postgres - 3Y RI</t>
   </si>
   <si>
+    <t>Formula / notes</t>
+  </si>
+  <si>
+    <t>Modeled monthly cost (selected scenario)</t>
+  </si>
+  <si>
+    <t>from Cost_Breakdown</t>
+  </si>
+  <si>
+    <t>Required monthly revenue for 90% margin</t>
+  </si>
+  <si>
+    <t>revenue = cost/(1-margin)</t>
+  </si>
+  <si>
+    <t>Required monthly revenue for 95% margin</t>
+  </si>
+  <si>
+    <t>Scenario-adjusted Pro users</t>
+  </si>
+  <si>
+    <t>Pro active users in selected scenario</t>
+  </si>
+  <si>
+    <t>Scenario-adjusted Team users</t>
+  </si>
+  <si>
+    <t>Team active users in selected scenario</t>
+  </si>
+  <si>
+    <t>Total paying users (Pro+Team)</t>
+  </si>
+  <si>
+    <t>free tier excluded</t>
+  </si>
+  <si>
+    <t>editable in Inputs</t>
+  </si>
+  <si>
+    <t>Price denominator (Pro + Team*multiplier)</t>
+  </si>
+  <si>
+    <t>for solving two-tier pricing</t>
+  </si>
+  <si>
+    <t>Recommended Pro price @90% margin</t>
+  </si>
+  <si>
+    <t>monthly price per Pro user</t>
+  </si>
+  <si>
+    <t>Recommended Team price @90% margin</t>
+  </si>
+  <si>
+    <t>monthly price per Team user</t>
+  </si>
+  <si>
+    <t>Blended ARPU needed @90% margin</t>
+  </si>
+  <si>
+    <t>monthly revenue / paying user</t>
+  </si>
+  <si>
+    <t>Recommended Pro price @95% margin</t>
+  </si>
+  <si>
+    <t>Recommended Team price @95% margin</t>
+  </si>
+  <si>
+    <t>Blended ARPU needed @95% margin</t>
+  </si>
+  <si>
+    <t>Margin check @95 pricing</t>
+  </si>
+  <si>
+    <t>should approximate target margin</t>
+  </si>
+  <si>
     <t>Case</t>
   </si>
   <si>
@@ -678,6 +769,21 @@
   </si>
   <si>
     <t>Lowest modeled monthly cost</t>
+  </si>
+  <si>
+    <t>Required revenue @90% margin</t>
+  </si>
+  <si>
+    <t>monthly</t>
+  </si>
+  <si>
+    <t>Required revenue @95% margin</t>
+  </si>
+  <si>
+    <t>Recommended Pro price @95%</t>
+  </si>
+  <si>
+    <t>Recommended Team price @95%</t>
   </si>
   <si>
     <t>Best commitment strategy</t>
@@ -1187,7 +1293,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2001,6 +2107,62 @@
       </c>
       <c r="D54" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>110</v>
+      </c>
+      <c r="B57" t="s">
+        <v>111</v>
+      </c>
+      <c r="C57" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="D57" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>110</v>
+      </c>
+      <c r="B58" t="s">
+        <v>112</v>
+      </c>
+      <c r="C58" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="D58" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>110</v>
+      </c>
+      <c r="B59" t="s">
+        <v>113</v>
+      </c>
+      <c r="C59" s="2">
+        <v>4</v>
+      </c>
+      <c r="D59" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2027,10 +2189,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>41</v>
@@ -2042,15 +2204,15 @@
         <v>43</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C2" s="3">
         <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C13*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))*Inputs!C3</f>
@@ -2067,10 +2229,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C3" s="3">
         <f>C2*(1+Inputs!C8)</f>
@@ -2087,10 +2249,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C4" s="3">
         <f>C3*Inputs!C7</f>
@@ -2107,10 +2269,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C5" s="3">
         <f>C4*Inputs!C15*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
@@ -2127,10 +2289,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C6" s="3">
         <f>(C5*Inputs!C20)/1024</f>
@@ -2147,10 +2309,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C7" s="3">
         <f>C4*Inputs!C21</f>
@@ -2167,10 +2329,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C8" s="3">
         <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C22*IF(Inputs!C2="Low",Inputs!E28,IF(Inputs!C2="High",Inputs!E30,Inputs!E29))</f>
@@ -2187,10 +2349,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C9" s="3">
         <f>(C3*Inputs!C24)/(1024*1024)</f>
@@ -2207,10 +2369,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B10" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C10" s="3">
         <f>C3*Inputs!C25</f>
@@ -2227,10 +2389,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B11" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C11" s="3">
         <f>(Inputs!C12/1000)*Inputs!C14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
@@ -2247,19 +2409,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F12" s="3">
         <f>Inputs!C4*60*Inputs!C51*Inputs!C52*(1-Inputs!C53)</f>
@@ -2267,19 +2429,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F13" s="3">
         <f>MAX(1,ROUNDUP(F5/F12,0))</f>
@@ -2287,19 +2449,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" t="s">
         <v>139</v>
       </c>
-      <c r="C14" t="s">
-        <v>135</v>
-      </c>
       <c r="D14" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E14" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F14" s="3">
         <f>MAX(1,ROUNDUP((F11*Inputs!C5)/Inputs!C54,0))</f>
@@ -2307,19 +2469,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B15" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F15" s="3">
         <f>MAX(Inputs!C6,F13,F14)</f>
@@ -2345,24 +2507,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B2" t="s">
         <v>81</v>
@@ -2379,10 +2541,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C3">
         <v>889</v>
@@ -2396,10 +2558,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C4">
         <v>1718</v>
@@ -2413,10 +2575,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C5">
         <v>0.089</v>
@@ -2430,10 +2592,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B6" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C6">
         <v>468</v>
@@ -2447,10 +2609,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C7">
         <v>936</v>
@@ -2464,10 +2626,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C8">
         <v>0.115</v>
@@ -2481,10 +2643,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B9" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C9">
         <v>0.095</v>
@@ -2498,10 +2660,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B10" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C10">
         <v>0.0208</v>
@@ -2515,16 +2677,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B11" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C11">
         <v>0.05</v>
       </c>
       <c r="D11" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E11" t="s">
         <v>3</v>
@@ -2532,16 +2694,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C12">
         <v>0.004</v>
       </c>
       <c r="D12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E12" t="s">
         <v>3</v>
@@ -2552,7 +2714,7 @@
         <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C13">
         <v>0.045</v>
@@ -2569,13 +2731,13 @@
         <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C14">
         <v>0.00036</v>
       </c>
       <c r="D14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E14" t="s">
         <v>3</v>
@@ -2603,7 +2765,7 @@
         <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C16">
         <v>0.005</v>
@@ -2617,10 +2779,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C17">
         <v>5.2795</v>
@@ -2651,27 +2813,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C2" s="3">
         <f>Inputs!C33*Inputs!C4*Formulas!F15</f>
@@ -2685,10 +2847,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C3" s="3">
         <f>Inputs!C47*Inputs!C4</f>
@@ -2702,10 +2864,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C4" s="3">
         <f>Inputs!C48</f>
@@ -2719,10 +2881,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C5" s="3">
         <f>(Inputs!C38/36)*2</f>
@@ -2739,7 +2901,7 @@
         <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C6" s="3">
         <f>Inputs!C39*128</f>
@@ -2753,10 +2915,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C7" s="3">
         <f>Inputs!C40*128*Inputs!C9</f>
@@ -2770,10 +2932,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C8" s="3">
         <f>Inputs!C41*MAX(128,Formulas!F6*3)</f>
@@ -2790,7 +2952,7 @@
         <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C9" s="3">
         <f>Inputs!C42*(Formulas!F4/10000)</f>
@@ -2807,7 +2969,7 @@
         <v>95</v>
       </c>
       <c r="B10" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C10" s="3">
         <f>Inputs!C43*(Formulas!F7/10000)</f>
@@ -2821,10 +2983,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C11" s="3">
         <f>Inputs!C44*MAX(5,Formulas!F9*2)</f>
@@ -2841,7 +3003,7 @@
         <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C12" s="3">
         <f>Inputs!C45*(Formulas!F10/10000)</f>
@@ -2855,10 +3017,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B13" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C13" s="3">
         <f>Inputs!C46*Formulas!F8</f>
@@ -2872,10 +3034,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C14" s="1">
         <f>SUM(C2:C13)</f>
@@ -2884,7 +3046,7 @@
         <f>SUM(D2:D13)</f>
       </c>
       <c r="E14" s="1" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2905,24 +3067,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B2" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -2939,7 +3101,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B3" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15</f>
@@ -2956,7 +3118,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B4" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15</f>
@@ -2973,7 +3135,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B5" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2</f>
@@ -2990,7 +3152,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B6" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2</f>
@@ -3007,7 +3169,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B7" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2</f>
@@ -3024,7 +3186,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B8" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2</f>
@@ -3046,6 +3208,210 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="3">
+        <f>Cost_Breakdown!C14</f>
+      </c>
+      <c r="C2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3" s="3">
+        <f>B2/(1-Inputs!C57)</f>
+      </c>
+      <c r="C3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="3">
+        <f>B2/(1-Inputs!C58)</f>
+      </c>
+      <c r="C4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B6" s="3">
+        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))</f>
+      </c>
+      <c r="C6" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B7" s="3">
+        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))</f>
+      </c>
+      <c r="C7" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B8" s="3">
+        <f>B6+B7</f>
+      </c>
+      <c r="C8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" s="3">
+        <f>Inputs!C59</f>
+      </c>
+      <c r="C9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>217</v>
+      </c>
+      <c r="B10" s="3">
+        <f>B6 + (B7*B9)</f>
+      </c>
+      <c r="C10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="3">
+        <f>B3/B10</f>
+      </c>
+      <c r="C12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="3">
+        <f>B12*B9</f>
+      </c>
+      <c r="C13" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="3">
+        <f>B3/B8</f>
+      </c>
+      <c r="C14" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>225</v>
+      </c>
+      <c r="B16" s="3">
+        <f>B4/B10</f>
+      </c>
+      <c r="C16" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="3">
+        <f>B16*B9</f>
+      </c>
+      <c r="C17" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>227</v>
+      </c>
+      <c r="B18" s="3">
+        <f>B4/B8</f>
+      </c>
+      <c r="C18" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="3"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>228</v>
+      </c>
+      <c r="B20" s="3">
+        <f>IF((B16*B6+B17*B7)=0,0,1-(B2/(B16*B6+B17*B7)))</f>
+      </c>
+      <c r="C20" t="s">
+        <v>229</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -3057,16 +3423,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>201</v>
+        <v>231</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>202</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3085,7 +3451,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>203</v>
+        <v>233</v>
       </c>
       <c r="B3">
         <v>0.75</v>
@@ -3099,7 +3465,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>204</v>
+        <v>234</v>
       </c>
       <c r="B4">
         <v>1.25</v>
@@ -3113,7 +3479,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="B5">
         <v>1.5</v>
@@ -3131,9 +3497,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -3142,29 +3508,29 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>206</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>237</v>
       </c>
       <c r="B2" s="3">
         <f>Inputs!C2</f>
       </c>
       <c r="C2" t="s">
-        <v>208</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>239</v>
       </c>
       <c r="B3" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -3175,101 +3541,145 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="B4" s="3">
         <f>Cost_Breakdown!D14</f>
       </c>
       <c r="C4" t="s">
-        <v>211</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="B5" s="3">
         <f>Formulas!F15</f>
       </c>
       <c r="C5" t="s">
-        <v>213</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>214</v>
+        <v>244</v>
       </c>
       <c r="B6" s="3">
         <f>Formulas!F13</f>
       </c>
       <c r="C6" t="s">
-        <v>215</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>216</v>
+        <v>246</v>
       </c>
       <c r="B7" s="3">
         <f>Formulas!F14</f>
       </c>
       <c r="C7" t="s">
-        <v>217</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>218</v>
+        <v>248</v>
       </c>
       <c r="B8" s="3">
         <f>MIN(Commitment_Compare!B2:B8)</f>
       </c>
       <c r="C8" t="s">
-        <v>219</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>220</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>199</v>
+        <v>250</v>
+      </c>
+      <c r="B9" s="3">
+        <f>Pricing_Strategy!B3</f>
       </c>
       <c r="C9" t="s">
-        <v>221</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>222</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>223</v>
+        <v>252</v>
+      </c>
+      <c r="B10" s="3">
+        <f>Pricing_Strategy!B4</f>
       </c>
       <c r="C10" t="s">
-        <v>224</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>225</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>226</v>
+        <v>253</v>
+      </c>
+      <c r="B11" s="3">
+        <f>Pricing_Strategy!B16</f>
       </c>
       <c r="C11" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>228</v>
-      </c>
-      <c r="B12" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B12" s="3">
+        <f>Pricing_Strategy!B17</f>
+      </c>
+      <c r="C12" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>255</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="C13" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>257</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>260</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C15" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>263</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C12" t="s">
-        <v>229</v>
+      <c r="C16" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add conversion-based margin pricing mode to cost model
</commit_message>
<xml_diff>
--- a/exports/costs/azure-cost-model.xlsx
+++ b/exports/costs/azure-cost-model.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="283">
   <si>
     <t>Workbook</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-02-10T02:52:00.477Z</t>
+    <t>2026-02-10T02:55:10.193Z</t>
   </si>
   <si>
     <t>Region</t>
@@ -363,6 +363,24 @@
     <t>Team price multiplier vs Pro</t>
   </si>
   <si>
+    <t>Pricing mode</t>
+  </si>
+  <si>
+    <t>tier_counts</t>
+  </si>
+  <si>
+    <t>(tier_counts/conversion_based)</t>
+  </si>
+  <si>
+    <t>Conversion to Pro rate</t>
+  </si>
+  <si>
+    <t>fraction of total active users</t>
+  </si>
+  <si>
+    <t>Conversion to Team rate</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -663,10 +681,46 @@
     <t>Team active users in selected scenario</t>
   </si>
   <si>
-    <t>Total paying users (Pro+Team)</t>
+    <t>Total active users (all cohorts)</t>
+  </si>
+  <si>
+    <t>used by conversion mode</t>
+  </si>
+  <si>
+    <t>Conversion-mode Pro users</t>
+  </si>
+  <si>
+    <t>from conversion rate</t>
+  </si>
+  <si>
+    <t>Conversion-mode Team users</t>
+  </si>
+  <si>
+    <t>Tier-count mode paying users (Pro+Team)</t>
   </si>
   <si>
     <t>free tier excluded</t>
+  </si>
+  <si>
+    <t>Active pricing mode</t>
+  </si>
+  <si>
+    <t>tier_counts or conversion_based</t>
+  </si>
+  <si>
+    <t>Selected Pro users</t>
+  </si>
+  <si>
+    <t>users used for pricing solve</t>
+  </si>
+  <si>
+    <t>Selected Team users</t>
+  </si>
+  <si>
+    <t>Total paying users (selected mode)</t>
+  </si>
+  <si>
+    <t>for blended ARPU</t>
   </si>
   <si>
     <t>editable in Inputs</t>
@@ -1293,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2165,10 +2219,55 @@
         <v>32</v>
       </c>
     </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>110</v>
+      </c>
+      <c r="B60" t="s">
+        <v>114</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D60" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>110</v>
+      </c>
+      <c r="B61" t="s">
+        <v>117</v>
+      </c>
+      <c r="C61" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="D61" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>110</v>
+      </c>
+      <c r="B62" t="s">
+        <v>119</v>
+      </c>
+      <c r="C62" s="2">
+        <v>0.015</v>
+      </c>
+      <c r="D62" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" sqref="C2">
       <formula1>"Low,Base,High"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="C60">
+      <formula1>"tier_counts,conversion_based"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2189,10 +2288,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>41</v>
@@ -2204,15 +2303,15 @@
         <v>43</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C2" s="3">
         <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C13*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))*Inputs!C3</f>
@@ -2229,10 +2328,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C3" s="3">
         <f>C2*(1+Inputs!C8)</f>
@@ -2249,10 +2348,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C4" s="3">
         <f>C3*Inputs!C7</f>
@@ -2269,10 +2368,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C5" s="3">
         <f>C4*Inputs!C15*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
@@ -2289,10 +2388,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C6" s="3">
         <f>(C5*Inputs!C20)/1024</f>
@@ -2309,10 +2408,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C7" s="3">
         <f>C4*Inputs!C21</f>
@@ -2329,10 +2428,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C8" s="3">
         <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C22*IF(Inputs!C2="Low",Inputs!E28,IF(Inputs!C2="High",Inputs!E30,Inputs!E29))</f>
@@ -2349,10 +2448,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C9" s="3">
         <f>(C3*Inputs!C24)/(1024*1024)</f>
@@ -2369,10 +2468,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B10" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C10" s="3">
         <f>C3*Inputs!C25</f>
@@ -2389,10 +2488,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C11" s="3">
         <f>(Inputs!C12/1000)*Inputs!C14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
@@ -2409,19 +2508,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F12" s="3">
         <f>Inputs!C4*60*Inputs!C51*Inputs!C52*(1-Inputs!C53)</f>
@@ -2429,19 +2528,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B13" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D13" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E13" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F13" s="3">
         <f>MAX(1,ROUNDUP(F5/F12,0))</f>
@@ -2449,19 +2548,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B14" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D14" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E14" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F14" s="3">
         <f>MAX(1,ROUNDUP((F11*Inputs!C5)/Inputs!C54,0))</f>
@@ -2469,19 +2568,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B15" t="s">
+        <v>151</v>
+      </c>
+      <c r="C15" t="s">
         <v>145</v>
       </c>
-      <c r="C15" t="s">
-        <v>139</v>
-      </c>
       <c r="D15" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E15" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F15" s="3">
         <f>MAX(Inputs!C6,F13,F14)</f>
@@ -2507,24 +2606,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
         <v>81</v>
@@ -2541,10 +2640,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C3">
         <v>889</v>
@@ -2558,10 +2657,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B4" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C4">
         <v>1718</v>
@@ -2575,10 +2674,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B5" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C5">
         <v>0.089</v>
@@ -2592,10 +2691,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C6">
         <v>468</v>
@@ -2609,10 +2708,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B7" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C7">
         <v>936</v>
@@ -2626,10 +2725,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C8">
         <v>0.115</v>
@@ -2643,10 +2742,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C9">
         <v>0.095</v>
@@ -2660,10 +2759,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B10" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C10">
         <v>0.0208</v>
@@ -2677,16 +2776,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B11" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C11">
         <v>0.05</v>
       </c>
       <c r="D11" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E11" t="s">
         <v>3</v>
@@ -2694,16 +2793,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B12" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C12">
         <v>0.004</v>
       </c>
       <c r="D12" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E12" t="s">
         <v>3</v>
@@ -2714,7 +2813,7 @@
         <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C13">
         <v>0.045</v>
@@ -2731,13 +2830,13 @@
         <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C14">
         <v>0.00036</v>
       </c>
       <c r="D14" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E14" t="s">
         <v>3</v>
@@ -2765,7 +2864,7 @@
         <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C16">
         <v>0.005</v>
@@ -2779,10 +2878,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B17" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C17">
         <v>5.2795</v>
@@ -2813,27 +2912,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C2" s="3">
         <f>Inputs!C33*Inputs!C4*Formulas!F15</f>
@@ -2847,10 +2946,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C3" s="3">
         <f>Inputs!C47*Inputs!C4</f>
@@ -2864,10 +2963,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B4" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C4" s="3">
         <f>Inputs!C48</f>
@@ -2881,10 +2980,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B5" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C5" s="3">
         <f>(Inputs!C38/36)*2</f>
@@ -2901,7 +3000,7 @@
         <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C6" s="3">
         <f>Inputs!C39*128</f>
@@ -2915,10 +3014,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B7" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="C7" s="3">
         <f>Inputs!C40*128*Inputs!C9</f>
@@ -2932,10 +3031,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B8" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C8" s="3">
         <f>Inputs!C41*MAX(128,Formulas!F6*3)</f>
@@ -2952,7 +3051,7 @@
         <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C9" s="3">
         <f>Inputs!C42*(Formulas!F4/10000)</f>
@@ -2969,7 +3068,7 @@
         <v>95</v>
       </c>
       <c r="B10" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C10" s="3">
         <f>Inputs!C43*(Formulas!F7/10000)</f>
@@ -2983,10 +3082,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B11" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C11" s="3">
         <f>Inputs!C44*MAX(5,Formulas!F9*2)</f>
@@ -3003,7 +3102,7 @@
         <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C12" s="3">
         <f>Inputs!C45*(Formulas!F10/10000)</f>
@@ -3017,10 +3116,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B13" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C13" s="3">
         <f>Inputs!C46*Formulas!F8</f>
@@ -3034,10 +3133,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C14" s="1">
         <f>SUM(C2:C13)</f>
@@ -3046,7 +3145,7 @@
         <f>SUM(D2:D13)</f>
       </c>
       <c r="E14" s="1" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3067,24 +3166,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B2" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -3101,7 +3200,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B3" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15</f>
@@ -3118,7 +3217,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B4" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15</f>
@@ -3135,7 +3234,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B5" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2</f>
@@ -3152,7 +3251,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B6" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2</f>
@@ -3169,7 +3268,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B7" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2</f>
@@ -3186,7 +3285,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B8" s="3">
         <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2</f>
@@ -3209,7 +3308,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -3219,46 +3318,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B2" s="3">
         <f>Cost_Breakdown!C14</f>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B3" s="3">
         <f>B2/(1-Inputs!C57)</f>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B4" s="3">
         <f>B2/(1-Inputs!C58)</f>
       </c>
       <c r="C4" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
@@ -3266,143 +3365,220 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B6" s="3">
         <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))</f>
       </c>
       <c r="C6" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B7" s="3">
         <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))</f>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B8" s="3">
-        <f>B6+B7</f>
+        <f>((Inputs!C12+Inputs!D12+Inputs!E12)*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29)))</f>
       </c>
       <c r="C8" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>222</v>
       </c>
       <c r="B9" s="3">
-        <f>Inputs!C59</f>
+        <f>B8*Inputs!C61</f>
       </c>
       <c r="C9" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="B10" s="3">
-        <f>B6 + (B7*B9)</f>
+        <f>B8*Inputs!C62</f>
       </c>
       <c r="C10" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B11" s="3">
+        <f>B6+B7</f>
+      </c>
+      <c r="C11" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B12" s="3">
-        <f>B3/B10</f>
+        <f>Inputs!C60</f>
       </c>
       <c r="C12" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B13" s="3">
-        <f>B12*B9</f>
+        <f>IF(B12="conversion_based",B9,B6)</f>
       </c>
       <c r="C13" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B14" s="3">
-        <f>B3/B8</f>
+        <f>IF(B12="conversion_based",B10,B7)</f>
       </c>
       <c r="C14" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
+        <v>230</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B15" s="3">
+        <f>B13+B14</f>
+      </c>
+      <c r="C15" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>225</v>
+        <v>113</v>
       </c>
       <c r="B16" s="3">
-        <f>B4/B10</f>
+        <f>Inputs!C59</f>
       </c>
       <c r="C16" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B17" s="3">
-        <f>B16*B9</f>
+        <f>B13 + (B14*B16)</f>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>227</v>
-      </c>
-      <c r="B18" s="3">
-        <f>B4/B8</f>
-      </c>
-      <c r="C18" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="3"/>
+        <v>236</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="3"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>237</v>
+      </c>
+      <c r="B19" s="3">
+        <f>IF(B17=0,0,B3/B17)</f>
+      </c>
+      <c r="C19" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="B20" s="3">
-        <f>IF((B16*B6+B17*B7)=0,0,1-(B2/(B16*B6+B17*B7)))</f>
+        <f>B19*B16</f>
       </c>
       <c r="C20" t="s">
-        <v>229</v>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>241</v>
+      </c>
+      <c r="B21" s="3">
+        <f>IF(B15=0,0,B3/B15)</f>
+      </c>
+      <c r="C21" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="3"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>243</v>
+      </c>
+      <c r="B23" s="3">
+        <f>IF(B17=0,0,B4/B17)</f>
+      </c>
+      <c r="C23" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>244</v>
+      </c>
+      <c r="B24" s="3">
+        <f>B23*B16</f>
+      </c>
+      <c r="C24" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>245</v>
+      </c>
+      <c r="B25" s="3">
+        <f>IF(B15=0,0,B4/B15)</f>
+      </c>
+      <c r="C25" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="3"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>246</v>
+      </c>
+      <c r="B27" s="3">
+        <f>IF((B23*B13+B24*B14)=0,0,1-(B2/(B23*B13+B24*B14)))</f>
+      </c>
+      <c r="C27" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -3423,16 +3599,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3451,7 +3627,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="B3">
         <v>0.75</v>
@@ -3465,7 +3641,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
       <c r="B4">
         <v>1.25</v>
@@ -3479,7 +3655,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>235</v>
+        <v>253</v>
       </c>
       <c r="B5">
         <v>1.5</v>
@@ -3508,29 +3684,29 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="B2" s="3">
         <f>Inputs!C2</f>
       </c>
       <c r="C2" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
       <c r="B3" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -3541,145 +3717,145 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="B4" s="3">
         <f>Cost_Breakdown!D14</f>
       </c>
       <c r="C4" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="B5" s="3">
         <f>Formulas!F15</f>
       </c>
       <c r="C5" t="s">
-        <v>243</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="B6" s="3">
         <f>Formulas!F13</f>
       </c>
       <c r="C6" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="B7" s="3">
         <f>Formulas!F14</f>
       </c>
       <c r="C7" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="B8" s="3">
         <f>MIN(Commitment_Compare!B2:B8)</f>
       </c>
       <c r="C8" t="s">
-        <v>249</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="B9" s="3">
         <f>Pricing_Strategy!B3</f>
       </c>
       <c r="C9" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
       <c r="B10" s="3">
         <f>Pricing_Strategy!B4</f>
       </c>
       <c r="C10" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="B11" s="3">
-        <f>Pricing_Strategy!B16</f>
+        <f>Pricing_Strategy!B23</f>
       </c>
       <c r="C11" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="B12" s="3">
-        <f>Pricing_Strategy!B17</f>
+        <f>Pricing_Strategy!B24</f>
       </c>
       <c r="C12" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C13" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="C14" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
       <c r="C15" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expose infra constants as editable cost-model assumptions
</commit_message>
<xml_diff>
--- a/exports/costs/azure-cost-model.xlsx
+++ b/exports/costs/azure-cost-model.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="291">
   <si>
     <t>Workbook</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-02-10T02:55:10.193Z</t>
+    <t>2026-02-10T03:00:00.248Z</t>
   </si>
   <si>
     <t>Region</t>
@@ -138,12 +138,36 @@
     <t>DB backup multiplier</t>
   </si>
   <si>
+    <t>Infra sizing knobs</t>
+  </si>
+  <si>
+    <t>Knob</t>
+  </si>
+  <si>
+    <t>Postgres vCores</t>
+  </si>
+  <si>
+    <t>Postgres storage GB</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>Blob storage floor GB</t>
+  </si>
+  <si>
+    <t>Blob audio retention multiplier</t>
+  </si>
+  <si>
+    <t>Table storage minimum GB</t>
+  </si>
+  <si>
+    <t>Table DB growth multiplier</t>
+  </si>
+  <si>
     <t>Cohort</t>
   </si>
   <si>
-    <t>Knob</t>
-  </si>
-  <si>
     <t>Free</t>
   </si>
   <si>
@@ -579,19 +603,19 @@
     <t>pg_vcore_3yr_reserved * vcores / 36</t>
   </si>
   <si>
-    <t>pg_storage_rate * 128GB</t>
+    <t>pg_storage_rate * configured_pg_gb</t>
   </si>
   <si>
     <t>Postgres backup</t>
   </si>
   <si>
-    <t>pg_backup_rate * 128GB * backup_multiplier</t>
+    <t>pg_backup_rate * configured_pg_gb * backup_multiplier</t>
   </si>
   <si>
     <t>Blob storage</t>
   </si>
   <si>
-    <t>blob_rate * MAX(128, audio_gb * 3)</t>
+    <t>blob_rate * MAX(blob_floor_gb, audio_gb*retention_mult)</t>
   </si>
   <si>
     <t>write_rate * episodes/10k</t>
@@ -603,7 +627,7 @@
     <t>Table storage</t>
   </si>
   <si>
-    <t>table_rate * MAX(5, db_growth*2)</t>
+    <t>table_rate * MAX(table_min_gb, db_growth*table_mult)</t>
   </si>
   <si>
     <t>table_ops_rate * table_ops/10k</t>
@@ -1347,7 +1371,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1487,7 +1511,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
@@ -1495,501 +1519,487 @@
         <v>40</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="C13" s="2">
+        <v>128</v>
+      </c>
+      <c r="D13" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="1" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="2">
+        <v>128</v>
+      </c>
+      <c r="D14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="2">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="2">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="2">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="2">
-        <v>2000</v>
-      </c>
-      <c r="D12" s="2">
-        <v>500</v>
-      </c>
-      <c r="E12" s="2">
-        <v>80</v>
-      </c>
-      <c r="F12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="2">
-        <v>0.4</v>
-      </c>
-      <c r="D13" s="2">
-        <v>1.2</v>
-      </c>
-      <c r="E13" s="2">
-        <v>4</v>
-      </c>
-      <c r="F13" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="2">
-        <v>35</v>
-      </c>
-      <c r="D14" s="2">
-        <v>55</v>
-      </c>
-      <c r="E14" s="2">
-        <v>95</v>
-      </c>
-      <c r="F14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="2">
-        <v>6</v>
-      </c>
-      <c r="D15" s="2">
-        <v>10</v>
-      </c>
-      <c r="E15" s="2">
-        <v>14</v>
-      </c>
-      <c r="F15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="2">
-        <v>900</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1700</v>
-      </c>
-      <c r="E16" s="2">
-        <v>2500</v>
-      </c>
-      <c r="F16" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17" s="2">
-        <v>0.7</v>
-      </c>
-      <c r="D17" s="2">
-        <v>0.7</v>
-      </c>
-      <c r="E17" s="2">
-        <v>0.6</v>
-      </c>
-      <c r="F17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="D18" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="E18" s="2">
-        <v>0.25</v>
-      </c>
-      <c r="F18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B19" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="D19" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="E19" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="F19" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2">
-        <v>0.45</v>
+        <v>2000</v>
       </c>
       <c r="D20" s="2">
-        <v>0.45</v>
+        <v>500</v>
       </c>
       <c r="E20" s="2">
-        <v>0.45</v>
+        <v>80</v>
       </c>
       <c r="F20" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C21" s="2">
-        <v>2.2</v>
+        <v>0.4</v>
       </c>
       <c r="D21" s="2">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="E21" s="2">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C22" s="2">
-        <v>0.18</v>
+        <v>35</v>
       </c>
       <c r="D22" s="2">
-        <v>0.55</v>
+        <v>55</v>
       </c>
       <c r="E22" s="2">
-        <v>1.8</v>
+        <v>95</v>
       </c>
       <c r="F22" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="C23" s="2">
+        <v>6</v>
+      </c>
+      <c r="D23" s="2">
+        <v>10</v>
+      </c>
+      <c r="E23" s="2">
         <v>14</v>
       </c>
-      <c r="D23" s="2">
-        <v>18</v>
-      </c>
-      <c r="E23" s="2">
-        <v>26</v>
-      </c>
       <c r="F23" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2">
-        <v>12</v>
+        <v>900</v>
       </c>
       <c r="D24" s="2">
-        <v>16</v>
+        <v>1700</v>
       </c>
       <c r="E24" s="2">
-        <v>24</v>
+        <v>2500</v>
       </c>
       <c r="F24" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="E25" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="F25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D26" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="F26" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="F27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="2">
+        <v>0.45</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0.45</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0.45</v>
+      </c>
+      <c r="F28" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="2">
+        <v>2.2</v>
+      </c>
+      <c r="D29" s="2">
+        <v>2.8</v>
+      </c>
+      <c r="E29" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="F29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>72</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B30" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C30" s="2">
+        <v>0.18</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0.55</v>
+      </c>
+      <c r="E30" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="F30" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="2">
+        <v>14</v>
+      </c>
+      <c r="D31" s="2">
         <v>18</v>
       </c>
-      <c r="D25" s="2">
-        <v>28</v>
-      </c>
-      <c r="E25" s="2">
-        <v>42</v>
-      </c>
-      <c r="F25" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="E31" s="2">
+        <v>26</v>
+      </c>
+      <c r="F31" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E27" s="1" t="s">
+      <c r="B32" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>75</v>
-      </c>
-      <c r="B28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C28" s="2">
-        <v>0.7</v>
-      </c>
-      <c r="D28" s="2">
-        <v>0.75</v>
-      </c>
-      <c r="E28" s="2">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C32" s="2">
+        <v>12</v>
+      </c>
+      <c r="D32" s="2">
+        <v>16</v>
+      </c>
+      <c r="E32" s="2">
         <v>24</v>
       </c>
-      <c r="C29" s="2">
-        <v>1</v>
-      </c>
-      <c r="D29" s="2">
-        <v>1</v>
-      </c>
-      <c r="E29" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="2">
-        <v>1.6</v>
-      </c>
-      <c r="D30" s="2">
-        <v>1.4</v>
-      </c>
-      <c r="E30" s="2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+      <c r="F32" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="1" t="s">
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>80</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>79</v>
       </c>
       <c r="B33" t="s">
         <v>81</v>
       </c>
-      <c r="C33" s="3">
-        <v>0.172</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="C33" s="2">
+        <v>18</v>
+      </c>
+      <c r="D33" s="2">
+        <v>28</v>
+      </c>
+      <c r="E33" s="2">
+        <v>42</v>
+      </c>
+      <c r="F33" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>79</v>
-      </c>
-      <c r="B34" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C34" s="3">
-        <v>889</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="B35" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>79</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="D35" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C35" s="3">
-        <v>1718</v>
-      </c>
-      <c r="D35" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E35" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B36" t="s">
-        <v>86</v>
-      </c>
-      <c r="C36" s="3">
-        <v>0.089</v>
-      </c>
-      <c r="D36" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="C36" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="D36" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="E36" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B37" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" s="2">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2">
+        <v>1</v>
+      </c>
+      <c r="E37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="D38" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="E38" s="2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C37" s="3">
-        <v>468</v>
-      </c>
-      <c r="D37" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" t="s">
+      <c r="B40" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C38" s="3">
-        <v>936</v>
-      </c>
-      <c r="D38" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>79</v>
-      </c>
-      <c r="B39" t="s">
-        <v>89</v>
-      </c>
-      <c r="C39" s="3">
-        <v>0.115</v>
-      </c>
-      <c r="D39" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>79</v>
-      </c>
-      <c r="B40" t="s">
-        <v>91</v>
-      </c>
-      <c r="C40" s="3">
-        <v>0.095</v>
-      </c>
-      <c r="D40" t="s">
-        <v>90</v>
+      <c r="C40" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B41" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C41" s="3">
-        <v>0.0208</v>
+        <v>0.172</v>
       </c>
       <c r="D41" t="s">
         <v>90</v>
@@ -1997,41 +2007,41 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C42" s="3">
-        <v>0.05</v>
+        <v>889</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C43" s="3">
-        <v>0.004</v>
+        <v>1718</v>
       </c>
       <c r="D43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C44" s="3">
-        <v>0.045</v>
+        <v>0.089</v>
       </c>
       <c r="D44" t="s">
         <v>90</v>
@@ -2039,226 +2049,338 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C45" s="3">
-        <v>0.00036</v>
+        <v>468</v>
       </c>
       <c r="D45" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B46" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C46" s="3">
-        <v>0.04</v>
+        <v>936</v>
       </c>
       <c r="D46" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B47" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C47" s="3">
-        <v>0.005</v>
+        <v>0.115</v>
       </c>
       <c r="D47" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B48" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="3">
+        <v>0.095</v>
+      </c>
+      <c r="D48" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" t="s">
+        <v>100</v>
+      </c>
+      <c r="C49" s="3">
+        <v>0.0208</v>
+      </c>
+      <c r="D49" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>87</v>
+      </c>
+      <c r="B50" t="s">
         <v>101</v>
       </c>
-      <c r="C48" s="3">
-        <v>5.2795</v>
-      </c>
-      <c r="D48" t="s">
+      <c r="C50" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="D50" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" t="s">
         <v>103</v>
       </c>
-      <c r="B51" t="s">
-        <v>104</v>
-      </c>
-      <c r="C51" s="2">
-        <v>2.4</v>
+      <c r="C51" s="3">
+        <v>0.004</v>
       </c>
       <c r="D51" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
-      </c>
-      <c r="C52" s="2">
-        <v>0.75</v>
+        <v>104</v>
+      </c>
+      <c r="C52" s="3">
+        <v>0.045</v>
       </c>
       <c r="D52" t="s">
-        <v>36</v>
+        <v>98</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="B53" t="s">
-        <v>107</v>
-      </c>
-      <c r="C53" s="2">
-        <v>0.2</v>
+        <v>105</v>
+      </c>
+      <c r="C53" s="3">
+        <v>0.00036</v>
       </c>
       <c r="D53" t="s">
-        <v>36</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="B54" t="s">
+        <v>106</v>
+      </c>
+      <c r="C54" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="D54" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>87</v>
+      </c>
+      <c r="B55" t="s">
         <v>108</v>
       </c>
-      <c r="C54" s="2">
-        <v>120</v>
-      </c>
-      <c r="D54" t="s">
+      <c r="C55" s="3">
+        <v>0.005</v>
+      </c>
+      <c r="D55" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+      <c r="C56" s="3">
+        <v>5.2795</v>
+      </c>
+      <c r="D56" t="s">
         <v>110</v>
       </c>
-      <c r="B56" s="1" t="s">
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C58" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D58" s="1" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>110</v>
-      </c>
-      <c r="B57" t="s">
-        <v>111</v>
-      </c>
-      <c r="C57" s="2">
-        <v>0.9</v>
-      </c>
-      <c r="D57" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>110</v>
-      </c>
-      <c r="B58" t="s">
-        <v>112</v>
-      </c>
-      <c r="C58" s="2">
-        <v>0.95</v>
-      </c>
-      <c r="D58" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B59" t="s">
+        <v>112</v>
+      </c>
+      <c r="C59" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="D59" t="s">
         <v>113</v>
-      </c>
-      <c r="C59" s="2">
-        <v>4</v>
-      </c>
-      <c r="D59" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B60" t="s">
         <v>114</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>115</v>
+      <c r="C60" s="2">
+        <v>0.75</v>
       </c>
       <c r="D60" t="s">
-        <v>116</v>
+        <v>36</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B61" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C61" s="2">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="D61" t="s">
-        <v>118</v>
+        <v>36</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B62" t="s">
+        <v>116</v>
+      </c>
+      <c r="C62" s="2">
+        <v>120</v>
+      </c>
+      <c r="D62" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>118</v>
+      </c>
+      <c r="B65" t="s">
         <v>119</v>
       </c>
-      <c r="C62" s="2">
+      <c r="C65" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="D65" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>118</v>
+      </c>
+      <c r="B66" t="s">
+        <v>120</v>
+      </c>
+      <c r="C66" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="D66" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>118</v>
+      </c>
+      <c r="B67" t="s">
+        <v>121</v>
+      </c>
+      <c r="C67" s="2">
+        <v>4</v>
+      </c>
+      <c r="D67" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>118</v>
+      </c>
+      <c r="B68" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D68" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>118</v>
+      </c>
+      <c r="B69" t="s">
+        <v>125</v>
+      </c>
+      <c r="C69" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="D69" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>118</v>
+      </c>
+      <c r="B70" t="s">
+        <v>127</v>
+      </c>
+      <c r="C70" s="2">
         <v>0.015</v>
       </c>
-      <c r="D62" t="s">
-        <v>118</v>
+      <c r="D70" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -2266,7 +2388,7 @@
     <dataValidation type="list" sqref="C2">
       <formula1>"Low,Base,High"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C60">
+    <dataValidation type="list" sqref="C68">
       <formula1>"tier_counts,conversion_based"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2288,39 +2410,39 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C2" s="3">
-        <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C13*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))*Inputs!C3</f>
+        <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))*Inputs!C13*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))*Inputs!C3</f>
       </c>
       <c r="D2" s="3">
-        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!D13*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))*Inputs!C3</f>
+        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))*Inputs!D13*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))*Inputs!C3</f>
       </c>
       <c r="E2" s="3">
-        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!E13*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))*Inputs!C3</f>
+        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))*Inputs!E13*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))*Inputs!C3</f>
       </c>
       <c r="F2" s="3">
         <f>SUM(C2:E2)</f>
@@ -2328,10 +2450,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C3" s="3">
         <f>C2*(1+Inputs!C8)</f>
@@ -2348,10 +2470,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="C4" s="3">
         <f>C3*Inputs!C7</f>
@@ -2368,19 +2490,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C5" s="3">
-        <f>C4*Inputs!C15*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+        <f>C4*Inputs!C15*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))</f>
       </c>
       <c r="D5" s="3">
-        <f>D4*Inputs!D15*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+        <f>D4*Inputs!D15*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))</f>
       </c>
       <c r="E5" s="3">
-        <f>E4*Inputs!E15*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+        <f>E4*Inputs!E15*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))</f>
       </c>
       <c r="F5" s="3">
         <f>SUM(C5:E5)</f>
@@ -2388,10 +2510,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="B6" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="C6" s="3">
         <f>(C5*Inputs!C20)/1024</f>
@@ -2408,10 +2530,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C7" s="3">
         <f>C4*Inputs!C21</f>
@@ -2428,19 +2550,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C8" s="3">
-        <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!C22*IF(Inputs!C2="Low",Inputs!E28,IF(Inputs!C2="High",Inputs!E30,Inputs!E29))</f>
+        <f>Inputs!C12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))*Inputs!C22*IF(Inputs!C2="Low",Inputs!E36,IF(Inputs!C2="High",Inputs!E38,Inputs!E37))</f>
       </c>
       <c r="D8" s="3">
-        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!D22*IF(Inputs!C2="Low",Inputs!E28,IF(Inputs!C2="High",Inputs!E30,Inputs!E29))</f>
+        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))*Inputs!D22*IF(Inputs!C2="Low",Inputs!E36,IF(Inputs!C2="High",Inputs!E38,Inputs!E37))</f>
       </c>
       <c r="E8" s="3">
-        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))*Inputs!E22*IF(Inputs!C2="Low",Inputs!E28,IF(Inputs!C2="High",Inputs!E30,Inputs!E29))</f>
+        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))*Inputs!E22*IF(Inputs!C2="Low",Inputs!E36,IF(Inputs!C2="High",Inputs!E38,Inputs!E37))</f>
       </c>
       <c r="F8" s="3">
         <f>SUM(C8:E8)</f>
@@ -2448,10 +2570,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C9" s="3">
         <f>(C3*Inputs!C24)/(1024*1024)</f>
@@ -2468,10 +2590,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C10" s="3">
         <f>C3*Inputs!C25</f>
@@ -2488,19 +2610,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B11" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C11" s="3">
-        <f>(Inputs!C12/1000)*Inputs!C14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+        <f>(Inputs!C12/1000)*Inputs!C14*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))</f>
       </c>
       <c r="D11" s="3">
-        <f>(Inputs!D12/1000)*Inputs!D14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+        <f>(Inputs!D12/1000)*Inputs!D14*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))</f>
       </c>
       <c r="E11" s="3">
-        <f>(Inputs!E12/1000)*Inputs!E14*IF(Inputs!C2="Low",Inputs!D28,IF(Inputs!C2="High",Inputs!D30,Inputs!D29))</f>
+        <f>(Inputs!E12/1000)*Inputs!E14*IF(Inputs!C2="Low",Inputs!D36,IF(Inputs!C2="High",Inputs!D38,Inputs!D37))</f>
       </c>
       <c r="F11" s="3">
         <f>SUM(C11:E11)</f>
@@ -2508,39 +2630,39 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C12" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D12" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E12" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F12" s="3">
-        <f>Inputs!C4*60*Inputs!C51*Inputs!C52*(1-Inputs!C53)</f>
+        <f>Inputs!C4*60*Inputs!C59*Inputs!C60*(1-Inputs!C61)</f>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="C13" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D13" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E13" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F13" s="3">
         <f>MAX(1,ROUNDUP(F5/F12,0))</f>
@@ -2548,39 +2670,39 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B14" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C14" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D14" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E14" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F14" s="3">
-        <f>MAX(1,ROUNDUP((F11*Inputs!C5)/Inputs!C54,0))</f>
+        <f>MAX(1,ROUNDUP((F11*Inputs!C5)/Inputs!C62,0))</f>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B15" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="C15" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D15" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E15" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F15" s="3">
         <f>MAX(Inputs!C6,F13,F14)</f>
@@ -2606,33 +2728,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C2">
         <v>0.172</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -2640,16 +2762,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C3">
         <v>889</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
         <v>3</v>
@@ -2657,16 +2779,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C4">
         <v>1718</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
         <v>3</v>
@@ -2674,16 +2796,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B5" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C5">
         <v>0.089</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E5" t="s">
         <v>3</v>
@@ -2691,16 +2813,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C6">
         <v>468</v>
       </c>
       <c r="D6" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
         <v>3</v>
@@ -2708,16 +2830,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C7">
         <v>936</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
         <v>3</v>
@@ -2725,16 +2847,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C8">
         <v>0.115</v>
       </c>
       <c r="D8" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E8" t="s">
         <v>3</v>
@@ -2742,16 +2864,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B9" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="C9">
         <v>0.095</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E9" t="s">
         <v>3</v>
@@ -2759,16 +2881,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B10" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C10">
         <v>0.0208</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E10" t="s">
         <v>3</v>
@@ -2776,16 +2898,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C11">
         <v>0.05</v>
       </c>
       <c r="D11" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E11" t="s">
         <v>3</v>
@@ -2793,16 +2915,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B12" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C12">
         <v>0.004</v>
       </c>
       <c r="D12" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E12" t="s">
         <v>3</v>
@@ -2810,16 +2932,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="C13">
         <v>0.045</v>
       </c>
       <c r="D13" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E13" t="s">
         <v>3</v>
@@ -2827,16 +2949,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C14">
         <v>0.00036</v>
       </c>
       <c r="D14" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E14" t="s">
         <v>3</v>
@@ -2844,16 +2966,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B15" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C15">
         <v>0.04</v>
       </c>
       <c r="D15" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E15" t="s">
         <v>3</v>
@@ -2861,16 +2983,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="C16">
         <v>0.005</v>
       </c>
       <c r="D16" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E16" t="s">
         <v>3</v>
@@ -2878,16 +3000,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B17" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C17">
         <v>5.2795</v>
       </c>
       <c r="D17" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="E17" t="s">
         <v>3</v>
@@ -2912,33 +3034,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C2" s="3">
-        <f>Inputs!C33*Inputs!C4*Formulas!F15</f>
+        <f>Inputs!C41*Inputs!C4*Formulas!F15</f>
       </c>
       <c r="D2" s="3">
-        <f>Inputs!C33*Inputs!C4*Formulas!F15*12</f>
+        <f>Inputs!C41*Inputs!C4*Formulas!F15*12</f>
       </c>
       <c r="E2" s="3">
         <f>C2/SUM(C2:C13)</f>
@@ -2946,16 +3068,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C3" s="3">
-        <f>Inputs!C47*Inputs!C4</f>
+        <f>Inputs!C55*Inputs!C4</f>
       </c>
       <c r="D3" s="3">
-        <f>Inputs!C47*Inputs!C4*12</f>
+        <f>Inputs!C55*Inputs!C4*12</f>
       </c>
       <c r="E3" s="3">
         <f>C3/SUM(C2:C13)</f>
@@ -2963,16 +3085,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B4" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="C4" s="3">
-        <f>Inputs!C48</f>
+        <f>Inputs!C56</f>
       </c>
       <c r="D4" s="3">
-        <f>Inputs!C48*12</f>
+        <f>Inputs!C56*12</f>
       </c>
       <c r="E4" s="3">
         <f>C4/SUM(C2:C13)</f>
@@ -2980,16 +3102,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B5" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="C5" s="3">
-        <f>(Inputs!C38/36)*2</f>
+        <f>(Inputs!C46/36)*Inputs!C12</f>
       </c>
       <c r="D5" s="3">
-        <f>(Inputs!C38/36)*2*12</f>
+        <f>(Inputs!C46/36)*Inputs!C12*12</f>
       </c>
       <c r="E5" s="3">
         <f>C5/SUM(C2:C13)</f>
@@ -2997,16 +3119,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="C6" s="3">
-        <f>Inputs!C39*128</f>
+        <f>Inputs!C47*Inputs!C13</f>
       </c>
       <c r="D6" s="3">
-        <f>Inputs!C39*128*12</f>
+        <f>Inputs!C47*Inputs!C13*12</f>
       </c>
       <c r="E6" s="3">
         <f>C6/SUM(C2:C13)</f>
@@ -3014,16 +3136,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B7" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C7" s="3">
-        <f>Inputs!C40*128*Inputs!C9</f>
+        <f>Inputs!C48*Inputs!C13*Inputs!C9</f>
       </c>
       <c r="D7" s="3">
-        <f>Inputs!C40*128*Inputs!C9*12</f>
+        <f>Inputs!C48*Inputs!C13*Inputs!C9*12</f>
       </c>
       <c r="E7" s="3">
         <f>C7/SUM(C2:C13)</f>
@@ -3031,16 +3153,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B8" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="C8" s="3">
-        <f>Inputs!C41*MAX(128,Formulas!F6*3)</f>
+        <f>Inputs!C49*MAX(Inputs!C14,Formulas!F6*Inputs!C15)</f>
       </c>
       <c r="D8" s="3">
-        <f>Inputs!C41*MAX(128,Formulas!F6*3)*12</f>
+        <f>Inputs!C49*MAX(Inputs!C14,Formulas!F6*Inputs!C15)*12</f>
       </c>
       <c r="E8" s="3">
         <f>C8/SUM(C2:C13)</f>
@@ -3048,16 +3170,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="C9" s="3">
-        <f>Inputs!C42*(Formulas!F4/10000)</f>
+        <f>Inputs!C50*(Formulas!F4/10000)</f>
       </c>
       <c r="D9" s="3">
-        <f>Inputs!C42*(Formulas!F4/10000)*12</f>
+        <f>Inputs!C50*(Formulas!F4/10000)*12</f>
       </c>
       <c r="E9" s="3">
         <f>C9/SUM(C2:C13)</f>
@@ -3065,16 +3187,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="C10" s="3">
-        <f>Inputs!C43*(Formulas!F7/10000)</f>
+        <f>Inputs!C51*(Formulas!F7/10000)</f>
       </c>
       <c r="D10" s="3">
-        <f>Inputs!C43*(Formulas!F7/10000)*12</f>
+        <f>Inputs!C51*(Formulas!F7/10000)*12</f>
       </c>
       <c r="E10" s="3">
         <f>C10/SUM(C2:C13)</f>
@@ -3082,16 +3204,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B11" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="C11" s="3">
-        <f>Inputs!C44*MAX(5,Formulas!F9*2)</f>
+        <f>Inputs!C52*MAX(Inputs!C16,Formulas!F9*Inputs!C17)</f>
       </c>
       <c r="D11" s="3">
-        <f>Inputs!C44*MAX(5,Formulas!F9*2)*12</f>
+        <f>Inputs!C52*MAX(Inputs!C16,Formulas!F9*Inputs!C17)*12</f>
       </c>
       <c r="E11" s="3">
         <f>C11/SUM(C2:C13)</f>
@@ -3099,16 +3221,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B12" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="C12" s="3">
-        <f>Inputs!C45*(Formulas!F10/10000)</f>
+        <f>Inputs!C53*(Formulas!F10/10000)</f>
       </c>
       <c r="D12" s="3">
-        <f>Inputs!C45*(Formulas!F10/10000)*12</f>
+        <f>Inputs!C53*(Formulas!F10/10000)*12</f>
       </c>
       <c r="E12" s="3">
         <f>C12/SUM(C2:C13)</f>
@@ -3116,16 +3238,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B13" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="C13" s="3">
-        <f>Inputs!C46*Formulas!F8</f>
+        <f>Inputs!C54*Formulas!F8</f>
       </c>
       <c r="D13" s="3">
-        <f>Inputs!C46*Formulas!F8*12</f>
+        <f>Inputs!C54*Formulas!F8*12</f>
       </c>
       <c r="E13" s="3">
         <f>C13/SUM(C2:C13)</f>
@@ -3133,10 +3255,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C14" s="1">
         <f>SUM(C2:C13)</f>
@@ -3145,7 +3267,7 @@
         <f>SUM(D2:D13)</f>
       </c>
       <c r="E14" s="1" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -3166,24 +3288,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B2" s="3">
         <f>Cost_Breakdown!C14</f>
@@ -3200,104 +3322,104 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B3" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C42/12)*Formulas!F15</f>
       </c>
       <c r="C3" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C42/12)*Formulas!F15*12</f>
       </c>
       <c r="D3" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C42/12)*Formulas!F15)</f>
       </c>
       <c r="E3" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C34/12)*Formulas!F15))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C42/12)*Formulas!F15))/B2)</f>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="B4" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C43/36)*Formulas!F15</f>
       </c>
       <c r="C4" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C43/36)*Formulas!F15*12</f>
       </c>
       <c r="D4" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C43/36)*Formulas!F15)</f>
       </c>
       <c r="E4" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C35/36)*Formulas!F15))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 + (Inputs!C43/36)*Formulas!F15))/B2)</f>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B5" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C45/12)*Inputs!C12</f>
       </c>
       <c r="C5" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C45/12)*Inputs!C12*12</f>
       </c>
       <c r="D5" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C45/12)*Inputs!C12)</f>
       </c>
       <c r="E5" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C37/12)*2))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C45/12)*Inputs!C12))/B2)</f>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B6" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C46/36)*Inputs!C12</f>
       </c>
       <c r="C6" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C46/36)*Inputs!C12*12</f>
       </c>
       <c r="D6" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C46/36)*Inputs!C12)</f>
       </c>
       <c r="E6" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C38/36)*2))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C5 + (Inputs!C46/36)*Inputs!C12))/B2)</f>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B7" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C42/12)*Formulas!F15 + (Inputs!C45/12)*Inputs!C12</f>
       </c>
       <c r="C7" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C42/12)*Formulas!F15 + (Inputs!C45/12)*Inputs!C12*12</f>
       </c>
       <c r="D7" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C42/12)*Formulas!F15 + (Inputs!C45/12)*Inputs!C12)</f>
       </c>
       <c r="E7" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C34/12)*Formulas!F15 + (Inputs!C37/12)*2))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C42/12)*Formulas!F15 + (Inputs!C45/12)*Inputs!C12))/B2)</f>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B8" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C43/36)*Formulas!F15 + (Inputs!C46/36)*Inputs!C12</f>
       </c>
       <c r="C8" s="3">
-        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2*12</f>
+        <f>Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C43/36)*Formulas!F15 + (Inputs!C46/36)*Inputs!C12*12</f>
       </c>
       <c r="D8" s="3">
-        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2)</f>
+        <f>B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C43/36)*Formulas!F15 + (Inputs!C46/36)*Inputs!C12)</f>
       </c>
       <c r="E8" s="3">
-        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C35/36)*Formulas!F15 + (Inputs!C38/36)*2))/B2)</f>
+        <f>IF(B2=0,0,(B2-(Cost_Breakdown!C14 - Cost_Breakdown!C2 - Cost_Breakdown!C5 + (Inputs!C43/36)*Formulas!F15 + (Inputs!C46/36)*Inputs!C12))/B2)</f>
       </c>
     </row>
   </sheetData>
@@ -3318,46 +3440,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B2" s="3">
         <f>Cost_Breakdown!C14</f>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B3" s="3">
-        <f>B2/(1-Inputs!C57)</f>
+        <f>B2/(1-Inputs!C65)</f>
       </c>
       <c r="C3" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B4" s="3">
-        <f>B2/(1-Inputs!C58)</f>
+        <f>B2/(1-Inputs!C66)</f>
       </c>
       <c r="C4" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
@@ -3365,134 +3487,134 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B6" s="3">
-        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))</f>
+        <f>Inputs!D12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))</f>
       </c>
       <c r="C6" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="B7" s="3">
-        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29))</f>
+        <f>Inputs!E12*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37))</f>
       </c>
       <c r="C7" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="B8" s="3">
-        <f>((Inputs!C12+Inputs!D12+Inputs!E12)*IF(Inputs!C2="Low",Inputs!C28,IF(Inputs!C2="High",Inputs!C30,Inputs!C29)))</f>
+        <f>((Inputs!C12+Inputs!D12+Inputs!E12)*IF(Inputs!C2="Low",Inputs!C36,IF(Inputs!C2="High",Inputs!C38,Inputs!C37)))</f>
       </c>
       <c r="C8" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B9" s="3">
-        <f>B8*Inputs!C61</f>
+        <f>B8*Inputs!C69</f>
       </c>
       <c r="C9" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B10" s="3">
-        <f>B8*Inputs!C62</f>
+        <f>B8*Inputs!C70</f>
       </c>
       <c r="C10" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B11" s="3">
         <f>B6+B7</f>
       </c>
       <c r="C11" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B12" s="3">
-        <f>Inputs!C60</f>
+        <f>Inputs!C68</f>
       </c>
       <c r="C12" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B13" s="3">
         <f>IF(B12="conversion_based",B9,B6)</f>
       </c>
       <c r="C13" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="B14" s="3">
         <f>IF(B12="conversion_based",B10,B7)</f>
       </c>
       <c r="C14" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B15" s="3">
         <f>B13+B14</f>
       </c>
       <c r="C15" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B16" s="3">
-        <f>Inputs!C59</f>
+        <f>Inputs!C67</f>
       </c>
       <c r="C16" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B17" s="3">
         <f>B13 + (B14*B16)</f>
       </c>
       <c r="C17" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
@@ -3500,35 +3622,35 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B19" s="3">
         <f>IF(B17=0,0,B3/B17)</f>
       </c>
       <c r="C19" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B20" s="3">
         <f>B19*B16</f>
       </c>
       <c r="C20" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="B21" s="3">
         <f>IF(B15=0,0,B3/B15)</f>
       </c>
       <c r="C21" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
@@ -3536,35 +3658,35 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="B23" s="3">
         <f>IF(B17=0,0,B4/B17)</f>
       </c>
       <c r="C23" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B24" s="3">
         <f>B23*B16</f>
       </c>
       <c r="C24" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="B25" s="3">
         <f>IF(B15=0,0,B4/B15)</f>
       </c>
       <c r="C25" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
@@ -3572,13 +3694,13 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B27" s="3">
         <f>IF((B23*B13+B24*B14)=0,0,1-(B2/(B23*B13+B24*B14)))</f>
       </c>
       <c r="C27" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -3599,16 +3721,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3627,7 +3749,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="B3">
         <v>0.75</v>
@@ -3641,7 +3763,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="B4">
         <v>1.25</v>
@@ -3655,7 +3777,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="B5">
         <v>1.5</v>
@@ -3684,178 +3806,178 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B2" s="3">
         <f>Inputs!C2</f>
       </c>
       <c r="C2" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="B3" s="3">
         <f>Cost_Breakdown!C14</f>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B4" s="3">
         <f>Cost_Breakdown!D14</f>
       </c>
       <c r="C4" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B5" s="3">
         <f>Formulas!F15</f>
       </c>
       <c r="C5" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="B6" s="3">
         <f>Formulas!F13</f>
       </c>
       <c r="C6" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="B7" s="3">
         <f>Formulas!F14</f>
       </c>
       <c r="C7" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="B8" s="3">
         <f>MIN(Commitment_Compare!B2:B8)</f>
       </c>
       <c r="C8" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="B9" s="3">
         <f>Pricing_Strategy!B3</f>
       </c>
       <c r="C9" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B10" s="3">
         <f>Pricing_Strategy!B4</f>
       </c>
       <c r="C10" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="B11" s="3">
         <f>Pricing_Strategy!B23</f>
       </c>
       <c r="C11" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="B12" s="3">
         <f>Pricing_Strategy!B24</f>
       </c>
       <c r="C12" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C13" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="C14" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C15" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete markdown artifact pipeline and close milestone plan
</commit_message>
<xml_diff>
--- a/exports/costs/azure-cost-model.xlsx
+++ b/exports/costs/azure-cost-model.xlsx
@@ -24,13 +24,13 @@
     <t>Workbook</t>
   </si>
   <si>
-    <t>Azure Cost Model - ListenLater</t>
+    <t>Azure Cost Model - ArticlePod</t>
   </si>
   <si>
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-02-10T03:00:00.248Z</t>
+    <t>2026-02-15T00:29:43.234Z</t>
   </si>
   <si>
     <t>Region</t>

</xml_diff>

<commit_message>
Implement C01-C07 cost optimization and serverless mirror groundwork
</commit_message>
<xml_diff>
--- a/exports/costs/azure-cost-model.xlsx
+++ b/exports/costs/azure-cost-model.xlsx
@@ -30,7 +30,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-02-15T00:29:43.234Z</t>
+    <t>2026-03-08T01:36:34.718Z</t>
   </si>
   <si>
     <t>Region</t>
@@ -882,7 +882,7 @@
     <t>Architecture baseline</t>
   </si>
   <si>
-    <t>Standard_D4as_v5, General Purpose Ddsv4 (2 vCore equivalent), Blob Hot LRS</t>
+    <t>Standard_B2s, General Purpose Ddsv4 (2 vCore equivalent), Blob Hot LRS</t>
   </si>
   <si>
     <t>from infra/main.bicep</t>
@@ -1999,7 +1999,7 @@
         <v>89</v>
       </c>
       <c r="C41" s="3">
-        <v>0.172</v>
+        <v>0.0499</v>
       </c>
       <c r="D41" t="s">
         <v>90</v>
@@ -2013,7 +2013,7 @@
         <v>91</v>
       </c>
       <c r="C42" s="3">
-        <v>889</v>
+        <v>213</v>
       </c>
       <c r="D42" t="s">
         <v>92</v>
@@ -2027,7 +2027,7 @@
         <v>93</v>
       </c>
       <c r="C43" s="3">
-        <v>1718</v>
+        <v>500</v>
       </c>
       <c r="D43" t="s">
         <v>92</v>
@@ -2751,7 +2751,7 @@
         <v>89</v>
       </c>
       <c r="C2">
-        <v>0.172</v>
+        <v>0.0499</v>
       </c>
       <c r="D2" t="s">
         <v>90</v>
@@ -2768,7 +2768,7 @@
         <v>164</v>
       </c>
       <c r="C3">
-        <v>889</v>
+        <v>213</v>
       </c>
       <c r="D3" t="s">
         <v>92</v>
@@ -2785,7 +2785,7 @@
         <v>165</v>
       </c>
       <c r="C4">
-        <v>1718</v>
+        <v>500</v>
       </c>
       <c r="D4" t="s">
         <v>92</v>

</xml_diff>